<commit_message>
Regenerate category quality reports
</commit_message>
<xml_diff>
--- a/category_quality_metrics.xlsx
+++ b/category_quality_metrics.xlsx
@@ -9,7 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="category_ranking" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="disagreement_samples" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="illion_only_categories" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="finv_only_categories" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="disagreement_samples" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,12 +470,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
     <col width="27" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -789,44 +791,257 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>═══ 6. Counterparty 对比 ═══</t>
+          <t>═══ 6. 单边 Category 覆盖缺口分布 ═══</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>双方都有有效 Counterparty</t>
+          <t>illion 有、finv 无 Category</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>30,516</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr"/>
+          <t>10,129 / 41,996 = 24.12%</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>详见 illion_only_categories：按 illion category 分布</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
+          <t>finv 有、illion 无有效 Category</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>2,412 / 34,279 = 7.04%</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>详见 finv_only_categories：区分 illion 为空和 All Other Credits</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr"/>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>═══ 7. Counterparty 对比 ═══</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>双方都有有效 Counterparty</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>30,516</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
           <t>Counterparty 完全一致 (case-insensitive)</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>13,441 / 30,516 = 44.05%</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr"/>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>═══ 8. AI分析（严格不一致抽样） ═══</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>AI 抽样行数</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>590</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>仅针对严格不一致样本；不代表全量交易准确率</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>AI 成功解析</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>508 / 590 = 86.1%</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>以下 AI 判断占比均以成功解析行数为分母</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>illion 更准</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>333 / 508 = 65.55%</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>AI 判断 illion 的类别更准确</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>finv 更准</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>130 / 508 = 25.59%</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>AI 判断 finv 的类别更准确</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>双方都合理</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>34 / 508 = 6.69%</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>双方分类都可接受</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>双方都不对</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>9 / 508 = 1.77%</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>AI 判断两边分类均不准确</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>AI 不确定</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>2 / 508 = 0.39%</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>交易文本不足以判断</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>AI 失败（API/解析）</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>82 / 590 = 13.9%</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>未成功解析的 AI 返回</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>AI 生成 finv TODO</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>96</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>详见 disagreement_ai_analysis.xlsx 的 todos</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="9">
     <mergeCell ref="A13:C13"/>
     <mergeCell ref="A19:C19"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A31:C31"/>
     <mergeCell ref="A9:C9"/>
     <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A35:C35"/>
     <mergeCell ref="A4:C4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -896,7 +1111,7 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>finv对应top类别</t>
+          <t>finv不一致Top3类别</t>
         </is>
       </c>
     </row>
@@ -929,7 +1144,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>External Transfers(2933), Internal Transfer(801), Credit Card Repayments(15)</t>
+          <t>Internal Transfer (801, 95.2%), Credit Card Repayments (15, 1.8%), Non SACC Loans (8, 1.0%)</t>
         </is>
       </c>
     </row>
@@ -962,7 +1177,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>SACC Loans(284), Non SACC Loans(255)</t>
+          <t>Non SACC Loans (255, 100.0%)</t>
         </is>
       </c>
     </row>
@@ -995,7 +1210,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Groceries(1513), Retail(111), Dining Out(33)</t>
+          <t>Retail (111, 49.6%), Dining Out (33, 14.7%), Personal Care (27, 12.1%)</t>
         </is>
       </c>
     </row>
@@ -1028,7 +1243,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Non SACC Loans(7474), SACC Loans(179), External Transfers(26)</t>
+          <t>SACC Loans (179, 81.4%), External Transfers (26, 11.8%), Internal Transfer (15, 6.8%)</t>
         </is>
       </c>
     </row>
@@ -1061,7 +1276,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Gambling(165), Subscription TV(122), Retail(8)</t>
+          <t>Gambling (165, 93.8%), Retail (8, 4.5%), Internal Transfer (2, 1.1%)</t>
         </is>
       </c>
     </row>
@@ -1094,7 +1309,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Fees(143), Dishonours(80), Internal Transfer(26)</t>
+          <t>Fees (143, 83.1%), Internal Transfer (26, 15.1%), Gyms and other memberships (2, 1.2%)</t>
         </is>
       </c>
     </row>
@@ -1127,7 +1342,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Dining Out(837), Information(29), Personal Care(24)</t>
+          <t>Information (29, 22.3%), Personal Care (24, 18.5%), Entertainment (21, 16.2%)</t>
         </is>
       </c>
     </row>
@@ -1160,7 +1375,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Internal Transfer(9616), External Transfers(82), Credit Card Repayments(43)</t>
+          <t>External Transfers (82, 64.6%), Credit Card Repayments (43, 33.9%), Subscription TV (2, 1.6%)</t>
         </is>
       </c>
     </row>
@@ -1193,7 +1408,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>External Transfers(86), Wages(35), Internal Transfer(2)</t>
+          <t>External Transfers (86, 69.9%), Wages (35, 28.5%), Internal Transfer (2, 1.6%)</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1441,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Transport(675), Automotive(79), Wages(22)</t>
+          <t>Automotive (79, 68.7%), Wages (22, 19.1%), Health (8, 7.0%)</t>
         </is>
       </c>
     </row>
@@ -1259,7 +1474,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Gambling(945), Dining Out(73), External Transfers(20)</t>
+          <t>Dining Out (73, 69.5%), External Transfers (20, 19.0%), Information (5, 4.8%)</t>
         </is>
       </c>
     </row>
@@ -1292,7 +1507,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Fees(61), Non SACC Loans(8), Retail(4)</t>
+          <t>Fees (61, 81.3%), Non SACC Loans (8, 10.7%), Retail (4, 5.3%)</t>
         </is>
       </c>
     </row>
@@ -1325,7 +1540,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Insurance(40), Travel(26), Retail(13)</t>
+          <t>Travel (26, 38.2%), Retail (13, 19.1%), External Transfers (11, 16.2%)</t>
         </is>
       </c>
     </row>
@@ -1358,7 +1573,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Department Stores(166), Groceries(53), Retail(6)</t>
+          <t>Groceries (53, 85.5%), Retail (6, 9.7%), External Transfers (2, 3.2%)</t>
         </is>
       </c>
     </row>
@@ -1391,7 +1606,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Groceries(26), External Transfers(15), Utilities(12)</t>
+          <t>Groceries (26, 55.3%), External Transfers (15, 31.9%), Internal Transfer (4, 8.5%)</t>
         </is>
       </c>
     </row>
@@ -1424,7 +1639,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Retail(143), SACC Loans(11), Personal Care(10)</t>
+          <t>SACC Loans (11, 23.9%), Personal Care (10, 21.7%), Information (8, 17.4%)</t>
         </is>
       </c>
     </row>
@@ -1457,7 +1672,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Health(22), Information(18), Home Improvement(16)</t>
+          <t>Information (18, 40.0%), Home Improvement (16, 35.6%), Personal Care (5, 11.1%)</t>
         </is>
       </c>
     </row>
@@ -1490,7 +1705,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Gyms and other memberships(155), Fees(26), Information(7)</t>
+          <t>Fees (26, 63.4%), Information (7, 17.1%), Entertainment (3, 7.3%)</t>
         </is>
       </c>
     </row>
@@ -1523,7 +1738,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Wages(558), Automotive(31), External Transfers(6)</t>
+          <t>Automotive (31, 83.8%), External Transfers (6, 16.2%)</t>
         </is>
       </c>
     </row>
@@ -1556,7 +1771,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Automotive(229), Transport(8), External Transfers(8)</t>
+          <t>Transport (8, 29.6%), External Transfers (8, 29.6%), Personal Care (4, 14.8%)</t>
         </is>
       </c>
     </row>
@@ -1589,7 +1804,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Entertainment(35), Personal Care(10), Dining Out(5)</t>
+          <t>Personal Care (10, 52.6%), Dining Out (5, 26.3%), Gambling (2, 10.5%)</t>
         </is>
       </c>
     </row>
@@ -1622,7 +1837,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Credit Card Repayments(468), Internal Transfer(9), Non SACC Loans(1)</t>
+          <t>Internal Transfer (9, 90.0%), Non SACC Loans (1, 10.0%)</t>
         </is>
       </c>
     </row>
@@ -1655,7 +1870,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Fees(1903), Health(6), Non SACC Loans(3)</t>
+          <t>Health (6, 66.7%), Non SACC Loans (3, 33.3%)</t>
         </is>
       </c>
     </row>
@@ -1688,7 +1903,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Personal Care(11), Insurance(3), Retail(2)</t>
+          <t>Insurance (3, 37.5%), Retail (2, 25.0%), Dining Out (1, 12.5%)</t>
         </is>
       </c>
     </row>
@@ -1721,7 +1936,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Travel(48), Entertainment(3), Dining Out(2)</t>
+          <t>Entertainment (3, 37.5%), Dining Out (2, 25.0%), Transport (2, 25.0%)</t>
         </is>
       </c>
     </row>
@@ -1754,7 +1969,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Telecommunications(146), Retail(2), Internal Transfer(1)</t>
+          <t>Retail (2, 50.0%), Internal Transfer (1, 25.0%), External Transfers (1, 25.0%)</t>
         </is>
       </c>
     </row>
@@ -1787,7 +2002,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Centrelink(110), External Transfers(3)</t>
+          <t>External Transfers (3, 100.0%)</t>
         </is>
       </c>
     </row>
@@ -1820,7 +2035,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Internal Transfer(3)</t>
+          <t>Internal Transfer (3, 100.0%)</t>
         </is>
       </c>
     </row>
@@ -1853,7 +2068,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Debt Collection(112), Dishonours(2)</t>
+          <t>Dishonours (2, 100.0%)</t>
         </is>
       </c>
     </row>
@@ -1886,7 +2101,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Home Improvement(48), External Transfers(2)</t>
+          <t>External Transfers (2, 100.0%)</t>
         </is>
       </c>
     </row>
@@ -1919,7 +2134,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>External Transfers(1)</t>
+          <t>External Transfers (1, 100.0%)</t>
         </is>
       </c>
     </row>
@@ -1952,7 +2167,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Overdrawn(168)</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1985,7 +2200,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Pet Care(8)</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1995,6 +2210,1253 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>illion_category</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>缺口数</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>占illion单边缺口</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>illion有效总数</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>finv缺失率</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Dining Out</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>4099</v>
+      </c>
+      <c r="C2" t="n">
+        <v>40.5</v>
+      </c>
+      <c r="D2" t="n">
+        <v>5066</v>
+      </c>
+      <c r="E2" t="n">
+        <v>80.90000000000001</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Groceries</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1295</v>
+      </c>
+      <c r="C3" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="D3" t="n">
+        <v>3032</v>
+      </c>
+      <c r="E3" t="n">
+        <v>42.7</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Automotive</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>561</v>
+      </c>
+      <c r="C4" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="D4" t="n">
+        <v>817</v>
+      </c>
+      <c r="E4" t="n">
+        <v>68.7</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>External Transfers</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>489</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="D5" t="n">
+        <v>4263</v>
+      </c>
+      <c r="E5" t="n">
+        <v>11.5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>420</v>
+      </c>
+      <c r="C6" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>609</v>
+      </c>
+      <c r="E6" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>381</v>
+      </c>
+      <c r="C7" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1171</v>
+      </c>
+      <c r="E7" t="n">
+        <v>32.5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>330</v>
+      </c>
+      <c r="C8" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="D8" t="n">
+        <v>397</v>
+      </c>
+      <c r="E8" t="n">
+        <v>83.09999999999999</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Gambling</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>321</v>
+      </c>
+      <c r="C9" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1371</v>
+      </c>
+      <c r="E9" t="n">
+        <v>23.4</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Gyms and other memberships</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>316</v>
+      </c>
+      <c r="C10" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="D10" t="n">
+        <v>512</v>
+      </c>
+      <c r="E10" t="n">
+        <v>61.7</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Subscription TV</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>215</v>
+      </c>
+      <c r="C11" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>513</v>
+      </c>
+      <c r="E11" t="n">
+        <v>41.9</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Insurance</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>186</v>
+      </c>
+      <c r="C12" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="D12" t="n">
+        <v>294</v>
+      </c>
+      <c r="E12" t="n">
+        <v>63.3</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>165</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="D13" t="n">
+        <v>219</v>
+      </c>
+      <c r="E13" t="n">
+        <v>75.3</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Fees</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>161</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="D14" t="n">
+        <v>2073</v>
+      </c>
+      <c r="E14" t="n">
+        <v>7.8</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>158</v>
+      </c>
+      <c r="C15" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="D15" t="n">
+        <v>217</v>
+      </c>
+      <c r="E15" t="n">
+        <v>72.8</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Telecommunications</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>150</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D16" t="n">
+        <v>300</v>
+      </c>
+      <c r="E16" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Non SACC Loans</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>143</v>
+      </c>
+      <c r="C17" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="D17" t="n">
+        <v>7837</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>138</v>
+      </c>
+      <c r="C18" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="D18" t="n">
+        <v>194</v>
+      </c>
+      <c r="E18" t="n">
+        <v>71.09999999999999</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Personal Care</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>106</v>
+      </c>
+      <c r="C19" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" t="n">
+        <v>125</v>
+      </c>
+      <c r="E19" t="n">
+        <v>84.8</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Dishonours</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>80</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D20" t="n">
+        <v>332</v>
+      </c>
+      <c r="E20" t="n">
+        <v>24.1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Rent</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>79</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D21" t="n">
+        <v>202</v>
+      </c>
+      <c r="E21" t="n">
+        <v>39.1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Department Stores</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>70</v>
+      </c>
+      <c r="C22" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D22" t="n">
+        <v>298</v>
+      </c>
+      <c r="E22" t="n">
+        <v>23.5</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Wages</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>49</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D23" t="n">
+        <v>644</v>
+      </c>
+      <c r="E23" t="n">
+        <v>7.6</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>44</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D24" t="n">
+        <v>45</v>
+      </c>
+      <c r="E24" t="n">
+        <v>97.8</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Internal Transfer</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>42</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D25" t="n">
+        <v>9785</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Information</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>37</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D26" t="n">
+        <v>113</v>
+      </c>
+      <c r="E26" t="n">
+        <v>32.7</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Donations</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>32</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D27" t="n">
+        <v>35</v>
+      </c>
+      <c r="E27" t="n">
+        <v>91.40000000000001</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Debt Collection</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>24</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D28" t="n">
+        <v>138</v>
+      </c>
+      <c r="E28" t="n">
+        <v>17.4</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Pet Care</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>12</v>
+      </c>
+      <c r="C29" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D29" t="n">
+        <v>20</v>
+      </c>
+      <c r="E29" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Centrelink</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>12</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D30" t="n">
+        <v>125</v>
+      </c>
+      <c r="E30" t="n">
+        <v>9.6</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Home Improvement</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>10</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D31" t="n">
+        <v>60</v>
+      </c>
+      <c r="E31" t="n">
+        <v>16.7</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Credit Card Repayments</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>4</v>
+      </c>
+      <c r="C32" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" t="n">
+        <v>482</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="27" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>finv_category</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>缺口数</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>占finv单边缺口</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>finv有效总数</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>illion无效率</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>illion为空</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>illion为All Other Credits</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>967</v>
+      </c>
+      <c r="C2" t="n">
+        <v>40.1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1265</v>
+      </c>
+      <c r="E2" t="n">
+        <v>76.40000000000001</v>
+      </c>
+      <c r="F2" t="n">
+        <v>965</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Non SACC Loans</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>533</v>
+      </c>
+      <c r="C3" t="n">
+        <v>22.1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>8294</v>
+      </c>
+      <c r="E3" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="F3" t="n">
+        <v>533</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>External Transfers</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>407</v>
+      </c>
+      <c r="C4" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="D4" t="n">
+        <v>3617</v>
+      </c>
+      <c r="E4" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="F4" t="n">
+        <v>128</v>
+      </c>
+      <c r="G4" t="n">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Dining Out</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>122</v>
+      </c>
+      <c r="C5" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1079</v>
+      </c>
+      <c r="E5" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="F5" t="n">
+        <v>120</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Wages</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>85</v>
+      </c>
+      <c r="C6" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D6" t="n">
+        <v>720</v>
+      </c>
+      <c r="E6" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="F6" t="n">
+        <v>63</v>
+      </c>
+      <c r="G6" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Home Improvement</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>64</v>
+      </c>
+      <c r="C7" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="D7" t="n">
+        <v>154</v>
+      </c>
+      <c r="E7" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="F7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G7" t="n">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Gambling</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>50</v>
+      </c>
+      <c r="C8" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1166</v>
+      </c>
+      <c r="E8" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="F8" t="n">
+        <v>50</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Gyms and other memberships</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>39</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="D9" t="n">
+        <v>198</v>
+      </c>
+      <c r="E9" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="F9" t="n">
+        <v>39</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Fees</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>32</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="D10" t="n">
+        <v>2168</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F10" t="n">
+        <v>32</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Groceries</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>28</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1626</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="F11" t="n">
+        <v>28</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Information</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>23</v>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="n">
+        <v>107</v>
+      </c>
+      <c r="E12" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="F12" t="n">
+        <v>23</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>15</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D13" t="n">
+        <v>77</v>
+      </c>
+      <c r="E13" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="F13" t="n">
+        <v>13</v>
+      </c>
+      <c r="G13" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Internal Transfer</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>12</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D14" t="n">
+        <v>10505</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F14" t="n">
+        <v>12</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>11</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D15" t="n">
+        <v>711</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F15" t="n">
+        <v>11</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Automotive</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>6</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D16" t="n">
+        <v>356</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="F16" t="n">
+        <v>6</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Personal Care</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>4</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D17" t="n">
+        <v>97</v>
+      </c>
+      <c r="E17" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="F17" t="n">
+        <v>4</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>3</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D18" t="n">
+        <v>17</v>
+      </c>
+      <c r="E18" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="F18" t="n">
+        <v>3</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>3</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D19" t="n">
+        <v>85</v>
+      </c>
+      <c r="E19" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F19" t="n">
+        <v>3</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>3</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D20" t="n">
+        <v>42</v>
+      </c>
+      <c r="E20" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="F20" t="n">
+        <v>3</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Department Stores</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>2</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D21" t="n">
+        <v>172</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F21" t="n">
+        <v>2</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Credit Card Repayments</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>2</v>
+      </c>
+      <c r="C22" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D22" t="n">
+        <v>528</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F22" t="n">
+        <v>2</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Insurance</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" t="n">
+        <v>50</v>
+      </c>
+      <c r="E23" t="n">
+        <v>2</v>
+      </c>
+      <c r="F23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>